<commit_message>
test/excel: Excel for Windows on lines/files (second run) and lines/held, cell for cell as Excel for Mac; the fit cases colformat sent again (the column's format shown); meta seconds of the fit files as they were
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/win/lines/files/typed-crossing.xlsx
+++ b/test/excel/win/lines/files/typed-crossing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xlcalc\work\lines-files-53320-1\out\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xlcalc\work\lines-files-8146-1\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19CE7990-27D1-42D0-BA77-BD05D050B50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE7DA526-0F46-4C66-AA72-2F45953B08ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>